<commit_message>
UI fixes: navbar mobile + spacing under nav
</commit_message>
<xml_diff>
--- a/1XW_TradeBlotter_Web.xlsx
+++ b/1XW_TradeBlotter_Web.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a601c1c2ba3d9f4/Trading/The Strategy Project/1XW Website/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="13_ncr:1_{6F5069F1-F0E7-4440-AA6D-4AFA11BBED1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A834F952-FDCD-4925-A9A9-BF13E3D8F658}"/>
+  <xr:revisionPtr revIDLastSave="161" documentId="13_ncr:1_{6F5069F1-F0E7-4440-AA6D-4AFA11BBED1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED251AEA-9BD5-42B6-BFF0-1E71639FD1C2}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blotter" sheetId="3" r:id="rId1"/>
@@ -1320,7 +1320,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1555,6 +1555,9 @@
     </xf>
     <xf numFmtId="22" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -2618,10 +2621,10 @@
                 <c:formatCode>d\-mmm\-yy</c:formatCode>
                 <c:ptCount val="52"/>
                 <c:pt idx="0">
-                  <c:v>46060</c:v>
+                  <c:v>46088</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46067</c:v>
+                  <c:v>46095</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8737,7 +8740,9 @@
       </c>
     </row>
     <row r="3" spans="2:28" x14ac:dyDescent="0.4">
-      <c r="B3" s="39"/>
+      <c r="B3" s="40">
+        <v>46081</v>
+      </c>
       <c r="C3" s="5">
         <v>0</v>
       </c>
@@ -8756,7 +8761,9 @@
         <v>1000000</v>
       </c>
       <c r="K3" s="16"/>
-      <c r="L3" s="15"/>
+      <c r="L3" s="94">
+        <v>0</v>
+      </c>
       <c r="M3" s="15">
         <f>H3</f>
         <v>0</v>
@@ -8769,7 +8776,10 @@
         <v>1000000</v>
       </c>
       <c r="P3" s="15"/>
-      <c r="R3" s="3">
+      <c r="Q3" s="94">
+        <v>0</v>
+      </c>
+      <c r="R3" s="94">
         <v>0</v>
       </c>
       <c r="T3" s="39"/>
@@ -8777,7 +8787,7 @@
     </row>
     <row r="4" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B4" s="40">
-        <v>46060</v>
+        <v>46088</v>
       </c>
       <c r="C4" s="5">
         <f>C3+1</f>
@@ -8842,7 +8852,7 @@
       </c>
       <c r="T4" s="40">
         <f>B4</f>
-        <v>46060</v>
+        <v>46088</v>
       </c>
       <c r="U4" s="5">
         <f>C4</f>
@@ -8855,7 +8865,7 @@
     <row r="5" spans="2:28" x14ac:dyDescent="0.4">
       <c r="B5" s="40">
         <f>B4+7</f>
-        <v>46067</v>
+        <v>46095</v>
       </c>
       <c r="C5" s="5">
         <f>C4+1</f>
@@ -8878,7 +8888,7 @@
       <c r="R5" s="3"/>
       <c r="T5" s="40">
         <f t="shared" ref="T5" si="1">B5</f>
-        <v>46067</v>
+        <v>46095</v>
       </c>
       <c r="U5" s="5">
         <f t="shared" ref="U5" si="2">C5</f>

</xml_diff>